<commit_message>
docs(razao): documentar saldos e fechamentos mensais
</commit_message>
<xml_diff>
--- a/modelo-razao-importacao.xlsx
+++ b/modelo-razao-importacao.xlsx
@@ -238,6 +238,76 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="A10" authorId="0" shapeId="0">
+      <text>
+        <t>Data do lancamento. Ex: 31/01/2024</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>Numero do lancamento, se existir. Pode ficar vazio.</t>
+      </text>
+    </comment>
+    <comment ref="C10" authorId="0" shapeId="0">
+      <text>
+        <t>Codigo reduzido da conta do bloco. Ex: 10001</t>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="0" shapeId="0">
+      <text>
+        <t>Classificacao completa. Ex: 1.1.01.01.01.10001</t>
+      </text>
+    </comment>
+    <comment ref="E10" authorId="0" shapeId="0">
+      <text>
+        <t>Nome da conta. Ex: CAIXA</t>
+      </text>
+    </comment>
+    <comment ref="F10" authorId="0" shapeId="0">
+      <text>
+        <t>Historico do lancamento</t>
+      </text>
+    </comment>
+    <comment ref="G10" authorId="0" shapeId="0">
+      <text>
+        <t>Codigo reduzido da conta de contrapartida. Ex: 20951</t>
+      </text>
+    </comment>
+    <comment ref="H10" authorId="0" shapeId="0">
+      <text>
+        <t>Valor a debito, se houver; preencha debito ou credito, nunca ambos.</t>
+      </text>
+    </comment>
+    <comment ref="I10" authorId="0" shapeId="0">
+      <text>
+        <t>Valor a credito, se houver; preencha debito ou credito, nunca ambos.</t>
+      </text>
+    </comment>
+    <comment ref="J10" authorId="0" shapeId="0">
+      <text>
+        <t>Saldo que abre a sequencia do exercicio no bloco. Opcional. Ex: 100,00D</t>
+      </text>
+    </comment>
+    <comment ref="K10" authorId="0" shapeId="0">
+      <text>
+        <t>Saldo observado da competencia mensal. Opcional. Ex: 1.256,68C</t>
+      </text>
+    </comment>
+    <comment ref="L10" authorId="0" shapeId="0">
+      <text>
+        <t>Saldo acumulado do exercicio. Opcional. Ex: 1.156,68C</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -529,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -541,7 +611,9 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -669,61 +741,33 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>saldo_exercicio_original</t>
+          <t>saldo_anterior</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>saldo</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>saldo_exercicio</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Data do lancamento. Ex: 31/01/2024</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Numero do lancamento, se existir. Pode ficar vazio.</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Codigo reduzido da conta do bloco. Ex: 10001</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Classificacao completa. Ex: 1.1.01.01.01.10001</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Nome da conta. Ex: CAIXA</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Historico do lancamento</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Codigo reduzido da conta de contrapartida. Ex: 20951</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>Valor a debito, se houver; preencha debito ou credito, nunca ambos.</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Valor a credito, se houver; preencha debito ou credito, nunca ambos.</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>Saldo do relatorio, opcional e apenas para conferencia. Ex: 1156,68C</t>
-        </is>
-      </c>
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -759,6 +803,16 @@
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
+          <t>100,00D</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>1.256,68C</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="inlineStr">
+        <is>
           <t>1156,68C</t>
         </is>
       </c>
@@ -795,7 +849,13 @@
       <c r="I13" s="11" t="n">
         <v>185</v>
       </c>
-      <c r="J13" s="11" t="inlineStr">
+      <c r="J13" s="11" t="n"/>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>1.441,68C</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>1341,68C</t>
         </is>
@@ -833,7 +893,13 @@
         <v>500</v>
       </c>
       <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="J14" s="11" t="n"/>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>500,00D</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>841,68C</t>
         </is>
@@ -850,6 +916,8 @@
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n"/>
       <c r="J15" s="11" t="n"/>
+      <c r="K15" s="11" t="n"/>
+      <c r="L15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -862,6 +930,8 @@
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n"/>
       <c r="J16" s="11" t="n"/>
+      <c r="K16" s="11" t="n"/>
+      <c r="L16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
@@ -874,6 +944,8 @@
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
       <c r="J17" s="11" t="n"/>
+      <c r="K17" s="11" t="n"/>
+      <c r="L17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -886,6 +958,8 @@
       <c r="H18" s="11" t="n"/>
       <c r="I18" s="11" t="n"/>
       <c r="J18" s="11" t="n"/>
+      <c r="K18" s="11" t="n"/>
+      <c r="L18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n"/>
@@ -898,6 +972,8 @@
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
       <c r="J19" s="11" t="n"/>
+      <c r="K19" s="11" t="n"/>
+      <c r="L19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -910,6 +986,8 @@
       <c r="H20" s="11" t="n"/>
       <c r="I20" s="11" t="n"/>
       <c r="J20" s="11" t="n"/>
+      <c r="K20" s="11" t="n"/>
+      <c r="L20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n"/>
@@ -922,6 +1000,8 @@
       <c r="H21" s="11" t="n"/>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -934,6 +1014,8 @@
       <c r="H22" s="11" t="n"/>
       <c r="I22" s="11" t="n"/>
       <c r="J22" s="11" t="n"/>
+      <c r="K22" s="11" t="n"/>
+      <c r="L22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n"/>
@@ -946,6 +1028,8 @@
       <c r="H23" s="11" t="n"/>
       <c r="I23" s="11" t="n"/>
       <c r="J23" s="11" t="n"/>
+      <c r="K23" s="11" t="n"/>
+      <c r="L23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -958,6 +1042,8 @@
       <c r="H24" s="11" t="n"/>
       <c r="I24" s="11" t="n"/>
       <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="n"/>
+      <c r="L24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n"/>
@@ -970,6 +1056,8 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
       <c r="J25" s="11" t="n"/>
+      <c r="K25" s="11" t="n"/>
+      <c r="L25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -982,6 +1070,8 @@
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="11" t="n"/>
       <c r="J26" s="11" t="n"/>
+      <c r="K26" s="11" t="n"/>
+      <c r="L26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n"/>
@@ -994,6 +1084,8 @@
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="11" t="n"/>
       <c r="J27" s="11" t="n"/>
+      <c r="K27" s="11" t="n"/>
+      <c r="L27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -1006,6 +1098,8 @@
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="11" t="n"/>
       <c r="J28" s="11" t="n"/>
+      <c r="K28" s="11" t="n"/>
+      <c r="L28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n"/>
@@ -1018,6 +1112,8 @@
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="11" t="n"/>
       <c r="J29" s="11" t="n"/>
+      <c r="K29" s="11" t="n"/>
+      <c r="L29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -1030,6 +1126,8 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="11" t="n"/>
       <c r="J30" s="11" t="n"/>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n"/>
@@ -1042,6 +1140,8 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="11" t="n"/>
       <c r="J31" s="11" t="n"/>
+      <c r="K31" s="11" t="n"/>
+      <c r="L31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -1054,6 +1154,8 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n"/>
       <c r="J32" s="11" t="n"/>
+      <c r="K32" s="11" t="n"/>
+      <c r="L32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -1066,6 +1168,8 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="11" t="n"/>
       <c r="J33" s="11" t="n"/>
+      <c r="K33" s="11" t="n"/>
+      <c r="L33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -1078,6 +1182,8 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="11" t="n"/>
       <c r="J34" s="11" t="n"/>
+      <c r="K34" s="11" t="n"/>
+      <c r="L34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n"/>
@@ -1090,6 +1196,8 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="11" t="n"/>
       <c r="J35" s="11" t="n"/>
+      <c r="K35" s="11" t="n"/>
+      <c r="L35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -1102,6 +1210,8 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="11" t="n"/>
       <c r="J36" s="11" t="n"/>
+      <c r="K36" s="11" t="n"/>
+      <c r="L36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n"/>
@@ -1114,6 +1224,8 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="11" t="n"/>
       <c r="J37" s="11" t="n"/>
+      <c r="K37" s="11" t="n"/>
+      <c r="L37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -1126,6 +1238,8 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="11" t="n"/>
       <c r="J38" s="11" t="n"/>
+      <c r="K38" s="11" t="n"/>
+      <c r="L38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n"/>
@@ -1138,6 +1252,8 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="11" t="n"/>
       <c r="J39" s="11" t="n"/>
+      <c r="K39" s="11" t="n"/>
+      <c r="L39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -1150,6 +1266,8 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="11" t="n"/>
       <c r="J40" s="11" t="n"/>
+      <c r="K40" s="11" t="n"/>
+      <c r="L40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n"/>
@@ -1162,6 +1280,8 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="11" t="n"/>
       <c r="J41" s="11" t="n"/>
+      <c r="K41" s="11" t="n"/>
+      <c r="L41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -1174,6 +1294,8 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="11" t="n"/>
       <c r="J42" s="11" t="n"/>
+      <c r="K42" s="11" t="n"/>
+      <c r="L42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n"/>
@@ -1186,6 +1308,8 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="11" t="n"/>
       <c r="J43" s="11" t="n"/>
+      <c r="K43" s="11" t="n"/>
+      <c r="L43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -1198,6 +1322,8 @@
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="11" t="n"/>
       <c r="J44" s="11" t="n"/>
+      <c r="K44" s="11" t="n"/>
+      <c r="L44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n"/>
@@ -1210,6 +1336,8 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="11" t="n"/>
       <c r="J45" s="11" t="n"/>
+      <c r="K45" s="11" t="n"/>
+      <c r="L45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -1222,6 +1350,8 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="11" t="n"/>
       <c r="J46" s="11" t="n"/>
+      <c r="K46" s="11" t="n"/>
+      <c r="L46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="n"/>
@@ -1234,6 +1364,8 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="11" t="n"/>
       <c r="J47" s="11" t="n"/>
+      <c r="K47" s="11" t="n"/>
+      <c r="L47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -1246,6 +1378,8 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="11" t="n"/>
       <c r="J48" s="11" t="n"/>
+      <c r="K48" s="11" t="n"/>
+      <c r="L48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="n"/>
@@ -1258,6 +1392,8 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="11" t="n"/>
       <c r="J49" s="11" t="n"/>
+      <c r="K49" s="11" t="n"/>
+      <c r="L49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -1270,6 +1406,8 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="11" t="n"/>
       <c r="J50" s="11" t="n"/>
+      <c r="K50" s="11" t="n"/>
+      <c r="L50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="n"/>
@@ -1282,6 +1420,8 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="11" t="n"/>
       <c r="J51" s="11" t="n"/>
+      <c r="K51" s="11" t="n"/>
+      <c r="L51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n"/>
@@ -1294,6 +1434,8 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="11" t="n"/>
       <c r="J52" s="11" t="n"/>
+      <c r="K52" s="11" t="n"/>
+      <c r="L52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n"/>
@@ -1306,6 +1448,8 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="11" t="n"/>
       <c r="J53" s="11" t="n"/>
+      <c r="K53" s="11" t="n"/>
+      <c r="L53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -1318,6 +1462,8 @@
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="11" t="n"/>
       <c r="J54" s="11" t="n"/>
+      <c r="K54" s="11" t="n"/>
+      <c r="L54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="n"/>
@@ -1330,6 +1476,8 @@
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="11" t="n"/>
       <c r="J55" s="11" t="n"/>
+      <c r="K55" s="11" t="n"/>
+      <c r="L55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -1342,6 +1490,8 @@
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="11" t="n"/>
       <c r="J56" s="11" t="n"/>
+      <c r="K56" s="11" t="n"/>
+      <c r="L56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="n"/>
@@ -1354,6 +1504,8 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="11" t="n"/>
       <c r="J57" s="11" t="n"/>
+      <c r="K57" s="11" t="n"/>
+      <c r="L57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -1366,6 +1518,8 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="11" t="n"/>
       <c r="J58" s="11" t="n"/>
+      <c r="K58" s="11" t="n"/>
+      <c r="L58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="n"/>
@@ -1378,6 +1532,8 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="11" t="n"/>
       <c r="J59" s="11" t="n"/>
+      <c r="K59" s="11" t="n"/>
+      <c r="L59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n"/>
@@ -1390,6 +1546,8 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="11" t="n"/>
       <c r="J60" s="11" t="n"/>
+      <c r="K60" s="11" t="n"/>
+      <c r="L60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -1402,6 +1560,8 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="11" t="n"/>
       <c r="J61" s="11" t="n"/>
+      <c r="K61" s="11" t="n"/>
+      <c r="L61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n"/>
@@ -1414,6 +1574,8 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="11" t="n"/>
       <c r="J62" s="11" t="n"/>
+      <c r="K62" s="11" t="n"/>
+      <c r="L62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="n"/>
@@ -1426,6 +1588,8 @@
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="11" t="n"/>
       <c r="J63" s="11" t="n"/>
+      <c r="K63" s="11" t="n"/>
+      <c r="L63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n"/>
@@ -1438,6 +1602,8 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="11" t="n"/>
       <c r="J64" s="11" t="n"/>
+      <c r="K64" s="11" t="n"/>
+      <c r="L64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="n"/>
@@ -1450,6 +1616,8 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="11" t="n"/>
       <c r="J65" s="11" t="n"/>
+      <c r="K65" s="11" t="n"/>
+      <c r="L65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n"/>
@@ -1462,6 +1630,8 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="11" t="n"/>
       <c r="J66" s="11" t="n"/>
+      <c r="K66" s="11" t="n"/>
+      <c r="L66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="n"/>
@@ -1474,6 +1644,8 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="11" t="n"/>
       <c r="J67" s="11" t="n"/>
+      <c r="K67" s="11" t="n"/>
+      <c r="L67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n"/>
@@ -1486,6 +1658,8 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="11" t="n"/>
       <c r="J68" s="11" t="n"/>
+      <c r="K68" s="11" t="n"/>
+      <c r="L68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="n"/>
@@ -1498,6 +1672,8 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="11" t="n"/>
       <c r="J69" s="11" t="n"/>
+      <c r="K69" s="11" t="n"/>
+      <c r="L69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n"/>
@@ -1510,6 +1686,8 @@
       <c r="H70" s="11" t="n"/>
       <c r="I70" s="11" t="n"/>
       <c r="J70" s="11" t="n"/>
+      <c r="K70" s="11" t="n"/>
+      <c r="L70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="n"/>
@@ -1522,6 +1700,8 @@
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="11" t="n"/>
       <c r="J71" s="11" t="n"/>
+      <c r="K71" s="11" t="n"/>
+      <c r="L71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n"/>
@@ -1534,6 +1714,8 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="11" t="n"/>
       <c r="J72" s="11" t="n"/>
+      <c r="K72" s="11" t="n"/>
+      <c r="L72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="n"/>
@@ -1546,6 +1728,8 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="11" t="n"/>
       <c r="J73" s="11" t="n"/>
+      <c r="K73" s="11" t="n"/>
+      <c r="L73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n"/>
@@ -1558,6 +1742,8 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="11" t="n"/>
       <c r="J74" s="11" t="n"/>
+      <c r="K74" s="11" t="n"/>
+      <c r="L74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="n"/>
@@ -1570,6 +1756,8 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="11" t="n"/>
       <c r="J75" s="11" t="n"/>
+      <c r="K75" s="11" t="n"/>
+      <c r="L75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n"/>
@@ -1582,6 +1770,8 @@
       <c r="H76" s="11" t="n"/>
       <c r="I76" s="11" t="n"/>
       <c r="J76" s="11" t="n"/>
+      <c r="K76" s="11" t="n"/>
+      <c r="L76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="n"/>
@@ -1594,6 +1784,8 @@
       <c r="H77" s="11" t="n"/>
       <c r="I77" s="11" t="n"/>
       <c r="J77" s="11" t="n"/>
+      <c r="K77" s="11" t="n"/>
+      <c r="L77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n"/>
@@ -1606,6 +1798,8 @@
       <c r="H78" s="11" t="n"/>
       <c r="I78" s="11" t="n"/>
       <c r="J78" s="11" t="n"/>
+      <c r="K78" s="11" t="n"/>
+      <c r="L78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="n"/>
@@ -1618,6 +1812,8 @@
       <c r="H79" s="11" t="n"/>
       <c r="I79" s="11" t="n"/>
       <c r="J79" s="11" t="n"/>
+      <c r="K79" s="11" t="n"/>
+      <c r="L79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n"/>
@@ -1630,6 +1826,8 @@
       <c r="H80" s="11" t="n"/>
       <c r="I80" s="11" t="n"/>
       <c r="J80" s="11" t="n"/>
+      <c r="K80" s="11" t="n"/>
+      <c r="L80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="n"/>
@@ -1642,6 +1840,8 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="11" t="n"/>
       <c r="J81" s="11" t="n"/>
+      <c r="K81" s="11" t="n"/>
+      <c r="L81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n"/>
@@ -1654,6 +1854,8 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="11" t="n"/>
       <c r="J82" s="11" t="n"/>
+      <c r="K82" s="11" t="n"/>
+      <c r="L82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="n"/>
@@ -1666,6 +1868,8 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="11" t="n"/>
       <c r="J83" s="11" t="n"/>
+      <c r="K83" s="11" t="n"/>
+      <c r="L83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n"/>
@@ -1678,6 +1882,8 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="11" t="n"/>
       <c r="J84" s="11" t="n"/>
+      <c r="K84" s="11" t="n"/>
+      <c r="L84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="n"/>
@@ -1690,6 +1896,8 @@
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="11" t="n"/>
       <c r="J85" s="11" t="n"/>
+      <c r="K85" s="11" t="n"/>
+      <c r="L85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n"/>
@@ -1702,6 +1910,8 @@
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="11" t="n"/>
       <c r="J86" s="11" t="n"/>
+      <c r="K86" s="11" t="n"/>
+      <c r="L86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="n"/>
@@ -1714,6 +1924,8 @@
       <c r="H87" s="11" t="n"/>
       <c r="I87" s="11" t="n"/>
       <c r="J87" s="11" t="n"/>
+      <c r="K87" s="11" t="n"/>
+      <c r="L87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n"/>
@@ -1726,6 +1938,8 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="11" t="n"/>
       <c r="J88" s="11" t="n"/>
+      <c r="K88" s="11" t="n"/>
+      <c r="L88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="n"/>
@@ -1738,6 +1952,8 @@
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="11" t="n"/>
       <c r="J89" s="11" t="n"/>
+      <c r="K89" s="11" t="n"/>
+      <c r="L89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n"/>
@@ -1750,6 +1966,8 @@
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="11" t="n"/>
       <c r="J90" s="11" t="n"/>
+      <c r="K90" s="11" t="n"/>
+      <c r="L90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="n"/>
@@ -1762,6 +1980,8 @@
       <c r="H91" s="11" t="n"/>
       <c r="I91" s="11" t="n"/>
       <c r="J91" s="11" t="n"/>
+      <c r="K91" s="11" t="n"/>
+      <c r="L91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n"/>
@@ -1774,6 +1994,8 @@
       <c r="H92" s="11" t="n"/>
       <c r="I92" s="11" t="n"/>
       <c r="J92" s="11" t="n"/>
+      <c r="K92" s="11" t="n"/>
+      <c r="L92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="n"/>
@@ -1786,6 +2008,8 @@
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="11" t="n"/>
       <c r="J93" s="11" t="n"/>
+      <c r="K93" s="11" t="n"/>
+      <c r="L93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n"/>
@@ -1798,6 +2022,8 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="11" t="n"/>
       <c r="J94" s="11" t="n"/>
+      <c r="K94" s="11" t="n"/>
+      <c r="L94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="n"/>
@@ -1810,6 +2036,8 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="11" t="n"/>
       <c r="J95" s="11" t="n"/>
+      <c r="K95" s="11" t="n"/>
+      <c r="L95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n"/>
@@ -1822,6 +2050,8 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="11" t="n"/>
       <c r="J96" s="11" t="n"/>
+      <c r="K96" s="11" t="n"/>
+      <c r="L96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="n"/>
@@ -1834,6 +2064,8 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="11" t="n"/>
       <c r="J97" s="11" t="n"/>
+      <c r="K97" s="11" t="n"/>
+      <c r="L97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n"/>
@@ -1846,6 +2078,8 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="11" t="n"/>
       <c r="J98" s="11" t="n"/>
+      <c r="K98" s="11" t="n"/>
+      <c r="L98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="n"/>
@@ -1858,6 +2092,8 @@
       <c r="H99" s="11" t="n"/>
       <c r="I99" s="11" t="n"/>
       <c r="J99" s="11" t="n"/>
+      <c r="K99" s="11" t="n"/>
+      <c r="L99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n"/>
@@ -1870,6 +2106,8 @@
       <c r="H100" s="11" t="n"/>
       <c r="I100" s="11" t="n"/>
       <c r="J100" s="11" t="n"/>
+      <c r="K100" s="11" t="n"/>
+      <c r="L100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="n"/>
@@ -1882,6 +2120,8 @@
       <c r="H101" s="11" t="n"/>
       <c r="I101" s="11" t="n"/>
       <c r="J101" s="11" t="n"/>
+      <c r="K101" s="11" t="n"/>
+      <c r="L101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n"/>
@@ -1894,6 +2134,8 @@
       <c r="H102" s="11" t="n"/>
       <c r="I102" s="11" t="n"/>
       <c r="J102" s="11" t="n"/>
+      <c r="K102" s="11" t="n"/>
+      <c r="L102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="n"/>
@@ -1906,6 +2148,8 @@
       <c r="H103" s="11" t="n"/>
       <c r="I103" s="11" t="n"/>
       <c r="J103" s="11" t="n"/>
+      <c r="K103" s="11" t="n"/>
+      <c r="L103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="n"/>
@@ -1918,6 +2162,8 @@
       <c r="H104" s="11" t="n"/>
       <c r="I104" s="11" t="n"/>
       <c r="J104" s="11" t="n"/>
+      <c r="K104" s="11" t="n"/>
+      <c r="L104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="n"/>
@@ -1930,6 +2176,8 @@
       <c r="H105" s="11" t="n"/>
       <c r="I105" s="11" t="n"/>
       <c r="J105" s="11" t="n"/>
+      <c r="K105" s="11" t="n"/>
+      <c r="L105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="n"/>
@@ -1942,6 +2190,8 @@
       <c r="H106" s="11" t="n"/>
       <c r="I106" s="11" t="n"/>
       <c r="J106" s="11" t="n"/>
+      <c r="K106" s="11" t="n"/>
+      <c r="L106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="n"/>
@@ -1954,6 +2204,8 @@
       <c r="H107" s="11" t="n"/>
       <c r="I107" s="11" t="n"/>
       <c r="J107" s="11" t="n"/>
+      <c r="K107" s="11" t="n"/>
+      <c r="L107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="n"/>
@@ -1966,6 +2218,8 @@
       <c r="H108" s="11" t="n"/>
       <c r="I108" s="11" t="n"/>
       <c r="J108" s="11" t="n"/>
+      <c r="K108" s="11" t="n"/>
+      <c r="L108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="n"/>
@@ -1978,6 +2232,8 @@
       <c r="H109" s="11" t="n"/>
       <c r="I109" s="11" t="n"/>
       <c r="J109" s="11" t="n"/>
+      <c r="K109" s="11" t="n"/>
+      <c r="L109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="n"/>
@@ -1990,6 +2246,8 @@
       <c r="H110" s="11" t="n"/>
       <c r="I110" s="11" t="n"/>
       <c r="J110" s="11" t="n"/>
+      <c r="K110" s="11" t="n"/>
+      <c r="L110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="n"/>
@@ -2002,6 +2260,8 @@
       <c r="H111" s="11" t="n"/>
       <c r="I111" s="11" t="n"/>
       <c r="J111" s="11" t="n"/>
+      <c r="K111" s="11" t="n"/>
+      <c r="L111" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -2032,6 +2292,7 @@
     <mergeCell ref="A8:J8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2041,7 +2302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2099,14 +2360,21 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>7. saldo_exercicio_original e opcional, serve apenas para conferencia e nao define debito/credito.</t>
+          <t>7. saldo_anterior abre o exercicio; saldo reinicia a cada mes; saldo_exercicio acumula o exercicio. Todos sao opcionais.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>8. Nao informe cod_dominio neste modelo. A importacao nao cria empresa automaticamente.</t>
+          <t>8. O alias antigo saldo_exercicio_original continua aceito como saldo_exercicio. Nao informe cod_dominio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9. Saldos sao para conferencia e fechamento; nao criam lancamento nem definem debito ou credito.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(razao): documentar saldos e fechamentos mensais (#541)
</commit_message>
<xml_diff>
--- a/modelo-razao-importacao.xlsx
+++ b/modelo-razao-importacao.xlsx
@@ -238,6 +238,76 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="A10" authorId="0" shapeId="0">
+      <text>
+        <t>Data do lancamento. Ex: 31/01/2024</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>Numero do lancamento, se existir. Pode ficar vazio.</t>
+      </text>
+    </comment>
+    <comment ref="C10" authorId="0" shapeId="0">
+      <text>
+        <t>Codigo reduzido da conta do bloco. Ex: 10001</t>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="0" shapeId="0">
+      <text>
+        <t>Classificacao completa. Ex: 1.1.01.01.01.10001</t>
+      </text>
+    </comment>
+    <comment ref="E10" authorId="0" shapeId="0">
+      <text>
+        <t>Nome da conta. Ex: CAIXA</t>
+      </text>
+    </comment>
+    <comment ref="F10" authorId="0" shapeId="0">
+      <text>
+        <t>Historico do lancamento</t>
+      </text>
+    </comment>
+    <comment ref="G10" authorId="0" shapeId="0">
+      <text>
+        <t>Codigo reduzido da conta de contrapartida. Ex: 20951</t>
+      </text>
+    </comment>
+    <comment ref="H10" authorId="0" shapeId="0">
+      <text>
+        <t>Valor a debito, se houver; preencha debito ou credito, nunca ambos.</t>
+      </text>
+    </comment>
+    <comment ref="I10" authorId="0" shapeId="0">
+      <text>
+        <t>Valor a credito, se houver; preencha debito ou credito, nunca ambos.</t>
+      </text>
+    </comment>
+    <comment ref="J10" authorId="0" shapeId="0">
+      <text>
+        <t>Saldo que abre a sequencia do exercicio no bloco. Opcional. Ex: 100,00D</t>
+      </text>
+    </comment>
+    <comment ref="K10" authorId="0" shapeId="0">
+      <text>
+        <t>Saldo observado da competencia mensal. Opcional. Ex: 1.256,68C</t>
+      </text>
+    </comment>
+    <comment ref="L10" authorId="0" shapeId="0">
+      <text>
+        <t>Saldo acumulado do exercicio. Opcional. Ex: 1.156,68C</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -529,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -541,7 +611,9 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -669,61 +741,33 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>saldo_exercicio_original</t>
+          <t>saldo_anterior</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>saldo</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>saldo_exercicio</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Data do lancamento. Ex: 31/01/2024</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Numero do lancamento, se existir. Pode ficar vazio.</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Codigo reduzido da conta do bloco. Ex: 10001</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Classificacao completa. Ex: 1.1.01.01.01.10001</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Nome da conta. Ex: CAIXA</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Historico do lancamento</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Codigo reduzido da conta de contrapartida. Ex: 20951</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>Valor a debito, se houver; preencha debito ou credito, nunca ambos.</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Valor a credito, se houver; preencha debito ou credito, nunca ambos.</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>Saldo do relatorio, opcional e apenas para conferencia. Ex: 1156,68C</t>
-        </is>
-      </c>
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -759,6 +803,16 @@
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
+          <t>100,00D</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>1.256,68C</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="inlineStr">
+        <is>
           <t>1156,68C</t>
         </is>
       </c>
@@ -795,7 +849,13 @@
       <c r="I13" s="11" t="n">
         <v>185</v>
       </c>
-      <c r="J13" s="11" t="inlineStr">
+      <c r="J13" s="11" t="n"/>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>1.441,68C</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>1341,68C</t>
         </is>
@@ -833,7 +893,13 @@
         <v>500</v>
       </c>
       <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="J14" s="11" t="n"/>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>500,00D</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>841,68C</t>
         </is>
@@ -850,6 +916,8 @@
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n"/>
       <c r="J15" s="11" t="n"/>
+      <c r="K15" s="11" t="n"/>
+      <c r="L15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -862,6 +930,8 @@
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n"/>
       <c r="J16" s="11" t="n"/>
+      <c r="K16" s="11" t="n"/>
+      <c r="L16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
@@ -874,6 +944,8 @@
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
       <c r="J17" s="11" t="n"/>
+      <c r="K17" s="11" t="n"/>
+      <c r="L17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -886,6 +958,8 @@
       <c r="H18" s="11" t="n"/>
       <c r="I18" s="11" t="n"/>
       <c r="J18" s="11" t="n"/>
+      <c r="K18" s="11" t="n"/>
+      <c r="L18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n"/>
@@ -898,6 +972,8 @@
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
       <c r="J19" s="11" t="n"/>
+      <c r="K19" s="11" t="n"/>
+      <c r="L19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -910,6 +986,8 @@
       <c r="H20" s="11" t="n"/>
       <c r="I20" s="11" t="n"/>
       <c r="J20" s="11" t="n"/>
+      <c r="K20" s="11" t="n"/>
+      <c r="L20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n"/>
@@ -922,6 +1000,8 @@
       <c r="H21" s="11" t="n"/>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -934,6 +1014,8 @@
       <c r="H22" s="11" t="n"/>
       <c r="I22" s="11" t="n"/>
       <c r="J22" s="11" t="n"/>
+      <c r="K22" s="11" t="n"/>
+      <c r="L22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n"/>
@@ -946,6 +1028,8 @@
       <c r="H23" s="11" t="n"/>
       <c r="I23" s="11" t="n"/>
       <c r="J23" s="11" t="n"/>
+      <c r="K23" s="11" t="n"/>
+      <c r="L23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -958,6 +1042,8 @@
       <c r="H24" s="11" t="n"/>
       <c r="I24" s="11" t="n"/>
       <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="n"/>
+      <c r="L24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n"/>
@@ -970,6 +1056,8 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
       <c r="J25" s="11" t="n"/>
+      <c r="K25" s="11" t="n"/>
+      <c r="L25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -982,6 +1070,8 @@
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="11" t="n"/>
       <c r="J26" s="11" t="n"/>
+      <c r="K26" s="11" t="n"/>
+      <c r="L26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n"/>
@@ -994,6 +1084,8 @@
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="11" t="n"/>
       <c r="J27" s="11" t="n"/>
+      <c r="K27" s="11" t="n"/>
+      <c r="L27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -1006,6 +1098,8 @@
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="11" t="n"/>
       <c r="J28" s="11" t="n"/>
+      <c r="K28" s="11" t="n"/>
+      <c r="L28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n"/>
@@ -1018,6 +1112,8 @@
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="11" t="n"/>
       <c r="J29" s="11" t="n"/>
+      <c r="K29" s="11" t="n"/>
+      <c r="L29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -1030,6 +1126,8 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="11" t="n"/>
       <c r="J30" s="11" t="n"/>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n"/>
@@ -1042,6 +1140,8 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="11" t="n"/>
       <c r="J31" s="11" t="n"/>
+      <c r="K31" s="11" t="n"/>
+      <c r="L31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -1054,6 +1154,8 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n"/>
       <c r="J32" s="11" t="n"/>
+      <c r="K32" s="11" t="n"/>
+      <c r="L32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -1066,6 +1168,8 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="11" t="n"/>
       <c r="J33" s="11" t="n"/>
+      <c r="K33" s="11" t="n"/>
+      <c r="L33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -1078,6 +1182,8 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="11" t="n"/>
       <c r="J34" s="11" t="n"/>
+      <c r="K34" s="11" t="n"/>
+      <c r="L34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n"/>
@@ -1090,6 +1196,8 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="11" t="n"/>
       <c r="J35" s="11" t="n"/>
+      <c r="K35" s="11" t="n"/>
+      <c r="L35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -1102,6 +1210,8 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="11" t="n"/>
       <c r="J36" s="11" t="n"/>
+      <c r="K36" s="11" t="n"/>
+      <c r="L36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n"/>
@@ -1114,6 +1224,8 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="11" t="n"/>
       <c r="J37" s="11" t="n"/>
+      <c r="K37" s="11" t="n"/>
+      <c r="L37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -1126,6 +1238,8 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="11" t="n"/>
       <c r="J38" s="11" t="n"/>
+      <c r="K38" s="11" t="n"/>
+      <c r="L38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n"/>
@@ -1138,6 +1252,8 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="11" t="n"/>
       <c r="J39" s="11" t="n"/>
+      <c r="K39" s="11" t="n"/>
+      <c r="L39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -1150,6 +1266,8 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="11" t="n"/>
       <c r="J40" s="11" t="n"/>
+      <c r="K40" s="11" t="n"/>
+      <c r="L40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n"/>
@@ -1162,6 +1280,8 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="11" t="n"/>
       <c r="J41" s="11" t="n"/>
+      <c r="K41" s="11" t="n"/>
+      <c r="L41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -1174,6 +1294,8 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="11" t="n"/>
       <c r="J42" s="11" t="n"/>
+      <c r="K42" s="11" t="n"/>
+      <c r="L42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n"/>
@@ -1186,6 +1308,8 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="11" t="n"/>
       <c r="J43" s="11" t="n"/>
+      <c r="K43" s="11" t="n"/>
+      <c r="L43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -1198,6 +1322,8 @@
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="11" t="n"/>
       <c r="J44" s="11" t="n"/>
+      <c r="K44" s="11" t="n"/>
+      <c r="L44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n"/>
@@ -1210,6 +1336,8 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="11" t="n"/>
       <c r="J45" s="11" t="n"/>
+      <c r="K45" s="11" t="n"/>
+      <c r="L45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -1222,6 +1350,8 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="11" t="n"/>
       <c r="J46" s="11" t="n"/>
+      <c r="K46" s="11" t="n"/>
+      <c r="L46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="n"/>
@@ -1234,6 +1364,8 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="11" t="n"/>
       <c r="J47" s="11" t="n"/>
+      <c r="K47" s="11" t="n"/>
+      <c r="L47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -1246,6 +1378,8 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="11" t="n"/>
       <c r="J48" s="11" t="n"/>
+      <c r="K48" s="11" t="n"/>
+      <c r="L48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="n"/>
@@ -1258,6 +1392,8 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="11" t="n"/>
       <c r="J49" s="11" t="n"/>
+      <c r="K49" s="11" t="n"/>
+      <c r="L49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -1270,6 +1406,8 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="11" t="n"/>
       <c r="J50" s="11" t="n"/>
+      <c r="K50" s="11" t="n"/>
+      <c r="L50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="n"/>
@@ -1282,6 +1420,8 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="11" t="n"/>
       <c r="J51" s="11" t="n"/>
+      <c r="K51" s="11" t="n"/>
+      <c r="L51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n"/>
@@ -1294,6 +1434,8 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="11" t="n"/>
       <c r="J52" s="11" t="n"/>
+      <c r="K52" s="11" t="n"/>
+      <c r="L52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n"/>
@@ -1306,6 +1448,8 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="11" t="n"/>
       <c r="J53" s="11" t="n"/>
+      <c r="K53" s="11" t="n"/>
+      <c r="L53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -1318,6 +1462,8 @@
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="11" t="n"/>
       <c r="J54" s="11" t="n"/>
+      <c r="K54" s="11" t="n"/>
+      <c r="L54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="n"/>
@@ -1330,6 +1476,8 @@
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="11" t="n"/>
       <c r="J55" s="11" t="n"/>
+      <c r="K55" s="11" t="n"/>
+      <c r="L55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -1342,6 +1490,8 @@
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="11" t="n"/>
       <c r="J56" s="11" t="n"/>
+      <c r="K56" s="11" t="n"/>
+      <c r="L56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="n"/>
@@ -1354,6 +1504,8 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="11" t="n"/>
       <c r="J57" s="11" t="n"/>
+      <c r="K57" s="11" t="n"/>
+      <c r="L57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -1366,6 +1518,8 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="11" t="n"/>
       <c r="J58" s="11" t="n"/>
+      <c r="K58" s="11" t="n"/>
+      <c r="L58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="n"/>
@@ -1378,6 +1532,8 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="11" t="n"/>
       <c r="J59" s="11" t="n"/>
+      <c r="K59" s="11" t="n"/>
+      <c r="L59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n"/>
@@ -1390,6 +1546,8 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="11" t="n"/>
       <c r="J60" s="11" t="n"/>
+      <c r="K60" s="11" t="n"/>
+      <c r="L60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -1402,6 +1560,8 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="11" t="n"/>
       <c r="J61" s="11" t="n"/>
+      <c r="K61" s="11" t="n"/>
+      <c r="L61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n"/>
@@ -1414,6 +1574,8 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="11" t="n"/>
       <c r="J62" s="11" t="n"/>
+      <c r="K62" s="11" t="n"/>
+      <c r="L62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="n"/>
@@ -1426,6 +1588,8 @@
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="11" t="n"/>
       <c r="J63" s="11" t="n"/>
+      <c r="K63" s="11" t="n"/>
+      <c r="L63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n"/>
@@ -1438,6 +1602,8 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="11" t="n"/>
       <c r="J64" s="11" t="n"/>
+      <c r="K64" s="11" t="n"/>
+      <c r="L64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="n"/>
@@ -1450,6 +1616,8 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="11" t="n"/>
       <c r="J65" s="11" t="n"/>
+      <c r="K65" s="11" t="n"/>
+      <c r="L65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n"/>
@@ -1462,6 +1630,8 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="11" t="n"/>
       <c r="J66" s="11" t="n"/>
+      <c r="K66" s="11" t="n"/>
+      <c r="L66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="n"/>
@@ -1474,6 +1644,8 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="11" t="n"/>
       <c r="J67" s="11" t="n"/>
+      <c r="K67" s="11" t="n"/>
+      <c r="L67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n"/>
@@ -1486,6 +1658,8 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="11" t="n"/>
       <c r="J68" s="11" t="n"/>
+      <c r="K68" s="11" t="n"/>
+      <c r="L68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="n"/>
@@ -1498,6 +1672,8 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="11" t="n"/>
       <c r="J69" s="11" t="n"/>
+      <c r="K69" s="11" t="n"/>
+      <c r="L69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n"/>
@@ -1510,6 +1686,8 @@
       <c r="H70" s="11" t="n"/>
       <c r="I70" s="11" t="n"/>
       <c r="J70" s="11" t="n"/>
+      <c r="K70" s="11" t="n"/>
+      <c r="L70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="n"/>
@@ -1522,6 +1700,8 @@
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="11" t="n"/>
       <c r="J71" s="11" t="n"/>
+      <c r="K71" s="11" t="n"/>
+      <c r="L71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n"/>
@@ -1534,6 +1714,8 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="11" t="n"/>
       <c r="J72" s="11" t="n"/>
+      <c r="K72" s="11" t="n"/>
+      <c r="L72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="n"/>
@@ -1546,6 +1728,8 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="11" t="n"/>
       <c r="J73" s="11" t="n"/>
+      <c r="K73" s="11" t="n"/>
+      <c r="L73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n"/>
@@ -1558,6 +1742,8 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="11" t="n"/>
       <c r="J74" s="11" t="n"/>
+      <c r="K74" s="11" t="n"/>
+      <c r="L74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="n"/>
@@ -1570,6 +1756,8 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="11" t="n"/>
       <c r="J75" s="11" t="n"/>
+      <c r="K75" s="11" t="n"/>
+      <c r="L75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n"/>
@@ -1582,6 +1770,8 @@
       <c r="H76" s="11" t="n"/>
       <c r="I76" s="11" t="n"/>
       <c r="J76" s="11" t="n"/>
+      <c r="K76" s="11" t="n"/>
+      <c r="L76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="n"/>
@@ -1594,6 +1784,8 @@
       <c r="H77" s="11" t="n"/>
       <c r="I77" s="11" t="n"/>
       <c r="J77" s="11" t="n"/>
+      <c r="K77" s="11" t="n"/>
+      <c r="L77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n"/>
@@ -1606,6 +1798,8 @@
       <c r="H78" s="11" t="n"/>
       <c r="I78" s="11" t="n"/>
       <c r="J78" s="11" t="n"/>
+      <c r="K78" s="11" t="n"/>
+      <c r="L78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="n"/>
@@ -1618,6 +1812,8 @@
       <c r="H79" s="11" t="n"/>
       <c r="I79" s="11" t="n"/>
       <c r="J79" s="11" t="n"/>
+      <c r="K79" s="11" t="n"/>
+      <c r="L79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n"/>
@@ -1630,6 +1826,8 @@
       <c r="H80" s="11" t="n"/>
       <c r="I80" s="11" t="n"/>
       <c r="J80" s="11" t="n"/>
+      <c r="K80" s="11" t="n"/>
+      <c r="L80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="n"/>
@@ -1642,6 +1840,8 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="11" t="n"/>
       <c r="J81" s="11" t="n"/>
+      <c r="K81" s="11" t="n"/>
+      <c r="L81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n"/>
@@ -1654,6 +1854,8 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="11" t="n"/>
       <c r="J82" s="11" t="n"/>
+      <c r="K82" s="11" t="n"/>
+      <c r="L82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="n"/>
@@ -1666,6 +1868,8 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="11" t="n"/>
       <c r="J83" s="11" t="n"/>
+      <c r="K83" s="11" t="n"/>
+      <c r="L83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n"/>
@@ -1678,6 +1882,8 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="11" t="n"/>
       <c r="J84" s="11" t="n"/>
+      <c r="K84" s="11" t="n"/>
+      <c r="L84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="n"/>
@@ -1690,6 +1896,8 @@
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="11" t="n"/>
       <c r="J85" s="11" t="n"/>
+      <c r="K85" s="11" t="n"/>
+      <c r="L85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n"/>
@@ -1702,6 +1910,8 @@
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="11" t="n"/>
       <c r="J86" s="11" t="n"/>
+      <c r="K86" s="11" t="n"/>
+      <c r="L86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="n"/>
@@ -1714,6 +1924,8 @@
       <c r="H87" s="11" t="n"/>
       <c r="I87" s="11" t="n"/>
       <c r="J87" s="11" t="n"/>
+      <c r="K87" s="11" t="n"/>
+      <c r="L87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n"/>
@@ -1726,6 +1938,8 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="11" t="n"/>
       <c r="J88" s="11" t="n"/>
+      <c r="K88" s="11" t="n"/>
+      <c r="L88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="n"/>
@@ -1738,6 +1952,8 @@
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="11" t="n"/>
       <c r="J89" s="11" t="n"/>
+      <c r="K89" s="11" t="n"/>
+      <c r="L89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n"/>
@@ -1750,6 +1966,8 @@
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="11" t="n"/>
       <c r="J90" s="11" t="n"/>
+      <c r="K90" s="11" t="n"/>
+      <c r="L90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="n"/>
@@ -1762,6 +1980,8 @@
       <c r="H91" s="11" t="n"/>
       <c r="I91" s="11" t="n"/>
       <c r="J91" s="11" t="n"/>
+      <c r="K91" s="11" t="n"/>
+      <c r="L91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n"/>
@@ -1774,6 +1994,8 @@
       <c r="H92" s="11" t="n"/>
       <c r="I92" s="11" t="n"/>
       <c r="J92" s="11" t="n"/>
+      <c r="K92" s="11" t="n"/>
+      <c r="L92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="n"/>
@@ -1786,6 +2008,8 @@
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="11" t="n"/>
       <c r="J93" s="11" t="n"/>
+      <c r="K93" s="11" t="n"/>
+      <c r="L93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n"/>
@@ -1798,6 +2022,8 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="11" t="n"/>
       <c r="J94" s="11" t="n"/>
+      <c r="K94" s="11" t="n"/>
+      <c r="L94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="n"/>
@@ -1810,6 +2036,8 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="11" t="n"/>
       <c r="J95" s="11" t="n"/>
+      <c r="K95" s="11" t="n"/>
+      <c r="L95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n"/>
@@ -1822,6 +2050,8 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="11" t="n"/>
       <c r="J96" s="11" t="n"/>
+      <c r="K96" s="11" t="n"/>
+      <c r="L96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="n"/>
@@ -1834,6 +2064,8 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="11" t="n"/>
       <c r="J97" s="11" t="n"/>
+      <c r="K97" s="11" t="n"/>
+      <c r="L97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n"/>
@@ -1846,6 +2078,8 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="11" t="n"/>
       <c r="J98" s="11" t="n"/>
+      <c r="K98" s="11" t="n"/>
+      <c r="L98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="n"/>
@@ -1858,6 +2092,8 @@
       <c r="H99" s="11" t="n"/>
       <c r="I99" s="11" t="n"/>
       <c r="J99" s="11" t="n"/>
+      <c r="K99" s="11" t="n"/>
+      <c r="L99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n"/>
@@ -1870,6 +2106,8 @@
       <c r="H100" s="11" t="n"/>
       <c r="I100" s="11" t="n"/>
       <c r="J100" s="11" t="n"/>
+      <c r="K100" s="11" t="n"/>
+      <c r="L100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="n"/>
@@ -1882,6 +2120,8 @@
       <c r="H101" s="11" t="n"/>
       <c r="I101" s="11" t="n"/>
       <c r="J101" s="11" t="n"/>
+      <c r="K101" s="11" t="n"/>
+      <c r="L101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n"/>
@@ -1894,6 +2134,8 @@
       <c r="H102" s="11" t="n"/>
       <c r="I102" s="11" t="n"/>
       <c r="J102" s="11" t="n"/>
+      <c r="K102" s="11" t="n"/>
+      <c r="L102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="n"/>
@@ -1906,6 +2148,8 @@
       <c r="H103" s="11" t="n"/>
       <c r="I103" s="11" t="n"/>
       <c r="J103" s="11" t="n"/>
+      <c r="K103" s="11" t="n"/>
+      <c r="L103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="n"/>
@@ -1918,6 +2162,8 @@
       <c r="H104" s="11" t="n"/>
       <c r="I104" s="11" t="n"/>
       <c r="J104" s="11" t="n"/>
+      <c r="K104" s="11" t="n"/>
+      <c r="L104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="n"/>
@@ -1930,6 +2176,8 @@
       <c r="H105" s="11" t="n"/>
       <c r="I105" s="11" t="n"/>
       <c r="J105" s="11" t="n"/>
+      <c r="K105" s="11" t="n"/>
+      <c r="L105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="n"/>
@@ -1942,6 +2190,8 @@
       <c r="H106" s="11" t="n"/>
       <c r="I106" s="11" t="n"/>
       <c r="J106" s="11" t="n"/>
+      <c r="K106" s="11" t="n"/>
+      <c r="L106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="n"/>
@@ -1954,6 +2204,8 @@
       <c r="H107" s="11" t="n"/>
       <c r="I107" s="11" t="n"/>
       <c r="J107" s="11" t="n"/>
+      <c r="K107" s="11" t="n"/>
+      <c r="L107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="n"/>
@@ -1966,6 +2218,8 @@
       <c r="H108" s="11" t="n"/>
       <c r="I108" s="11" t="n"/>
       <c r="J108" s="11" t="n"/>
+      <c r="K108" s="11" t="n"/>
+      <c r="L108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="n"/>
@@ -1978,6 +2232,8 @@
       <c r="H109" s="11" t="n"/>
       <c r="I109" s="11" t="n"/>
       <c r="J109" s="11" t="n"/>
+      <c r="K109" s="11" t="n"/>
+      <c r="L109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="n"/>
@@ -1990,6 +2246,8 @@
       <c r="H110" s="11" t="n"/>
       <c r="I110" s="11" t="n"/>
       <c r="J110" s="11" t="n"/>
+      <c r="K110" s="11" t="n"/>
+      <c r="L110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="n"/>
@@ -2002,6 +2260,8 @@
       <c r="H111" s="11" t="n"/>
       <c r="I111" s="11" t="n"/>
       <c r="J111" s="11" t="n"/>
+      <c r="K111" s="11" t="n"/>
+      <c r="L111" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -2032,6 +2292,7 @@
     <mergeCell ref="A8:J8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2041,7 +2302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2099,14 +2360,21 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>7. saldo_exercicio_original e opcional, serve apenas para conferencia e nao define debito/credito.</t>
+          <t>7. saldo_anterior abre o exercicio; saldo reinicia a cada mes; saldo_exercicio acumula o exercicio. Todos sao opcionais.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>8. Nao informe cod_dominio neste modelo. A importacao nao cria empresa automaticamente.</t>
+          <t>8. O alias antigo saldo_exercicio_original continua aceito como saldo_exercicio. Nao informe cod_dominio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9. Saldos sao para conferencia e fechamento; nao criam lancamento nem definem debito ou credito.</t>
         </is>
       </c>
     </row>

</xml_diff>